<commit_message>
Remove staff requested duty related data for 20260309-20260405
Remove staff requested duty related data for 20260309-20260405
</commit_message>
<xml_diff>
--- a/test/production/20260309-20260405/ward_requested_duty_excel.xlsx
+++ b/test/production/20260309-20260405/ward_requested_duty_excel.xlsx
@@ -294,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
@@ -312,6 +312,10 @@
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="3" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="4" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="4" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -989,8 +993,12 @@
       </c>
       <c r="U2"/>
       <c r="V2" s="11"/>
-      <c r="W2"/>
-      <c r="X2"/>
+      <c r="W2" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" t="s">
+        <v>39</v>
+      </c>
       <c r="Y2" s="10"/>
       <c r="Z2" s="10"/>
       <c r="AA2" s="10"/>
@@ -1003,7 +1011,9 @@
       <c r="AF2"/>
       <c r="AG2" s="10"/>
       <c r="AH2" s="10"/>
-      <c r="AI2" s="10"/>
+      <c r="AI2" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="AJ2" s="11"/>
       <c r="AK2" s="2"/>
     </row>
@@ -1030,6 +1040,9 @@
         <v>39</v>
       </c>
       <c r="H3" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
         <v>39</v>
       </c>
       <c r="J3" s="2"/>
@@ -1044,8 +1057,12 @@
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3" s="10"/>
-      <c r="T3" s="10"/>
-      <c r="U3"/>
+      <c r="T3" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" t="s">
+        <v>39</v>
+      </c>
       <c r="V3" s="11"/>
       <c r="W3"/>
       <c r="X3"/>
@@ -1103,7 +1120,9 @@
       <c r="R4" s="10"/>
       <c r="S4" s="10"/>
       <c r="T4" s="10"/>
-      <c r="U4"/>
+      <c r="U4" t="s">
+        <v>39</v>
+      </c>
       <c r="V4" s="11"/>
       <c r="W4"/>
       <c r="X4"/>
@@ -1112,8 +1131,12 @@
       <c r="AA4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AB4"/>
-      <c r="AC4" s="11"/>
+      <c r="AB4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC4" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="AD4"/>
       <c r="AE4"/>
       <c r="AF4"/>
@@ -1153,10 +1176,18 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="16"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
+      <c r="N5" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="O5" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="P5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
       <c r="T5" s="5"/>
@@ -1218,18 +1249,30 @@
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
       <c r="L6" s="9"/>
-      <c r="M6" s="2"/>
-      <c r="N6"/>
-      <c r="O6" s="1"/>
-      <c r="P6"/>
-      <c r="Q6"/>
+      <c r="M6" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="N6" t="s">
+        <v>39</v>
+      </c>
+      <c r="O6" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>39</v>
+      </c>
       <c r="R6"/>
       <c r="S6" s="10"/>
       <c r="T6" s="10"/>
       <c r="U6"/>
       <c r="V6" s="11"/>
       <c r="W6"/>
-      <c r="X6"/>
+      <c r="X6" t="s">
+        <v>38</v>
+      </c>
       <c r="Y6"/>
       <c r="Z6" s="10"/>
       <c r="AA6" s="2" t="s">
@@ -1329,8 +1372,13 @@
       <c r="H8" s="8" t="s">
         <v>40</v>
       </c>
+      <c r="I8" t="s">
+        <v>39</v>
+      </c>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="19" t="s">
+        <v>39</v>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8"/>
@@ -1344,10 +1392,14 @@
       <c r="V8" s="11"/>
       <c r="W8"/>
       <c r="X8" s="10"/>
-      <c r="Y8"/>
+      <c r="Y8" t="s">
+        <v>38</v>
+      </c>
       <c r="Z8" s="10"/>
       <c r="AA8" s="10"/>
-      <c r="AB8"/>
+      <c r="AB8" t="s">
+        <v>39</v>
+      </c>
       <c r="AC8" s="11"/>
       <c r="AD8" t="s">
         <v>41</v>
@@ -1404,11 +1456,21 @@
       <c r="Y9" s="5"/>
       <c r="Z9" s="5"/>
       <c r="AA9" s="5"/>
-      <c r="AB9" s="5"/>
-      <c r="AC9" s="6"/>
-      <c r="AD9" s="5"/>
-      <c r="AE9" s="5"/>
-      <c r="AF9" s="5"/>
+      <c r="AB9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF9" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="AG9" s="5" t="s">
         <v>41</v>
       </c>
@@ -1456,7 +1518,7 @@
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10"/>
-      <c r="O10" s="17"/>
+      <c r="O10" s="21"/>
       <c r="P10" s="10"/>
       <c r="Q10" s="10"/>
       <c r="R10" s="10"/>
@@ -1465,11 +1527,21 @@
       </c>
       <c r="T10" s="10"/>
       <c r="U10" s="10"/>
-      <c r="V10" s="11"/>
-      <c r="W10" s="10"/>
-      <c r="X10" s="10"/>
-      <c r="Y10" s="10"/>
-      <c r="Z10" s="10"/>
+      <c r="V10" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="W10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="X10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z10" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="AA10" s="10"/>
       <c r="AB10" s="10"/>
       <c r="AC10" s="11"/>
@@ -1482,8 +1554,8 @@
       <c r="AH10" s="10"/>
       <c r="AI10" s="10"/>
       <c r="AJ10" s="11"/>
-      <c r="AK10" s="18"/>
-      <c r="AL10" s="18"/>
+      <c r="AK10" s="22"/>
+      <c r="AL10" s="22"/>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
@@ -1512,9 +1584,15 @@
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="12"/>
+      <c r="L11" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="O11" s="1"/>
       <c r="P11"/>
       <c r="Q11"/>
@@ -1532,15 +1610,21 @@
       <c r="AA11" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AB11"/>
-      <c r="AC11" s="11"/>
+      <c r="AB11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC11" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="AD11"/>
       <c r="AE11"/>
       <c r="AF11"/>
       <c r="AG11" s="10"/>
       <c r="AH11" s="10"/>
       <c r="AI11"/>
-      <c r="AJ11" s="11"/>
+      <c r="AJ11" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="AK11" s="2"/>
     </row>
     <row r="12" ht="14.25">
@@ -1578,9 +1662,15 @@
       <c r="Q12" t="s">
         <v>41</v>
       </c>
-      <c r="R12"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="10"/>
+      <c r="R12" t="s">
+        <v>39</v>
+      </c>
+      <c r="S12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="T12" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="U12"/>
       <c r="V12" s="11"/>
       <c r="W12"/>
@@ -1592,8 +1682,12 @@
       </c>
       <c r="AB12"/>
       <c r="AC12" s="11"/>
-      <c r="AD12"/>
-      <c r="AE12"/>
+      <c r="AD12" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>39</v>
+      </c>
       <c r="AF12"/>
       <c r="AG12" s="10"/>
       <c r="AH12" s="10"/>
@@ -1637,8 +1731,12 @@
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
       <c r="T13" s="5"/>
-      <c r="U13" s="5"/>
-      <c r="V13" s="6"/>
+      <c r="U13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="V13" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="W13" s="5"/>
       <c r="X13" s="5"/>
       <c r="Y13" s="5"/>
@@ -1652,7 +1750,9 @@
       <c r="AG13" s="5"/>
       <c r="AH13" s="5"/>
       <c r="AI13" s="5"/>
-      <c r="AJ13" s="6"/>
+      <c r="AJ13" s="6" t="s">
+        <v>39</v>
+      </c>
       <c r="AK13" s="3"/>
     </row>
     <row r="14" ht="14.25">
@@ -1692,8 +1792,12 @@
       <c r="P14"/>
       <c r="Q14"/>
       <c r="R14"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="10"/>
+      <c r="S14" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="T14" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="U14"/>
       <c r="V14" s="11"/>
       <c r="W14"/>
@@ -1711,7 +1815,9 @@
       <c r="AE14"/>
       <c r="AF14"/>
       <c r="AG14" s="10"/>
-      <c r="AH14" s="10"/>
+      <c r="AH14" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="AI14"/>
       <c r="AJ14" s="11"/>
       <c r="AK14" s="2"/>
@@ -1742,12 +1848,24 @@
         <v>43</v>
       </c>
       <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="10"/>
+      <c r="K15" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="M15" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="N15" t="s">
+        <v>39</v>
+      </c>
+      <c r="O15" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="P15" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="Q15" s="10" t="s">
         <v>41</v>
       </c>
@@ -1772,8 +1890,8 @@
       <c r="AH15" s="10"/>
       <c r="AI15" s="10"/>
       <c r="AJ15" s="11"/>
-      <c r="AK15" s="18"/>
-      <c r="AL15" s="18"/>
+      <c r="AK15" s="22"/>
+      <c r="AL15" s="22"/>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" t="s">
@@ -1800,7 +1918,9 @@
       <c r="H16" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="2"/>
+      <c r="J16" s="19" t="s">
+        <v>39</v>
+      </c>
       <c r="K16" s="2"/>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -1821,10 +1941,18 @@
       <c r="Z16" s="10"/>
       <c r="AA16" s="10"/>
       <c r="AB16"/>
-      <c r="AC16" s="11"/>
-      <c r="AD16" s="10"/>
-      <c r="AE16"/>
-      <c r="AF16"/>
+      <c r="AC16" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD16" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE16" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF16" t="s">
+        <v>39</v>
+      </c>
       <c r="AG16" s="2" t="s">
         <v>41</v>
       </c>
@@ -1864,13 +1992,21 @@
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="16"/>
-      <c r="O17" s="19"/>
+      <c r="O17" s="23"/>
       <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="5"/>
-      <c r="S17" s="5"/>
+      <c r="Q17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="R17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S17" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="T17" s="5"/>
-      <c r="U17" s="5"/>
+      <c r="U17" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="V17" s="6"/>
       <c r="W17" s="5"/>
       <c r="X17" s="3" t="s">
@@ -1879,7 +2015,9 @@
       <c r="Y17" s="5"/>
       <c r="Z17" s="5"/>
       <c r="AA17" s="5"/>
-      <c r="AB17" s="5"/>
+      <c r="AB17" s="5" t="s">
+        <v>39</v>
+      </c>
       <c r="AC17" s="6"/>
       <c r="AD17" s="5"/>
       <c r="AE17" s="5"/>
@@ -1915,7 +2053,12 @@
       <c r="H18" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J18" s="2"/>
+      <c r="I18" t="s">
+        <v>39</v>
+      </c>
+      <c r="J18" s="19" t="s">
+        <v>39</v>
+      </c>
       <c r="K18" s="2"/>
       <c r="L18" s="2"/>
       <c r="M18" s="9"/>
@@ -1969,14 +2112,23 @@
       <c r="H19" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="2"/>
+      <c r="I19" t="s">
+        <v>39</v>
+      </c>
+      <c r="J19" s="19" t="s">
+        <v>39</v>
+      </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19"/>
       <c r="O19" s="1"/>
-      <c r="P19"/>
-      <c r="Q19"/>
+      <c r="P19" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>39</v>
+      </c>
       <c r="R19"/>
       <c r="S19" s="10"/>
       <c r="T19" s="10"/>
@@ -2033,18 +2185,30 @@
       <c r="Q20"/>
       <c r="R20"/>
       <c r="S20" s="10"/>
-      <c r="T20" s="10"/>
-      <c r="U20"/>
-      <c r="V20" s="11"/>
-      <c r="W20" s="10"/>
+      <c r="T20" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="U20" t="s">
+        <v>39</v>
+      </c>
+      <c r="V20" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="W20" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="X20"/>
       <c r="Y20"/>
       <c r="Z20" s="10"/>
       <c r="AA20" s="10"/>
       <c r="AB20"/>
       <c r="AC20" s="11"/>
-      <c r="AD20"/>
-      <c r="AE20"/>
+      <c r="AD20" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>39</v>
+      </c>
       <c r="AF20"/>
       <c r="AG20" s="10"/>
       <c r="AH20" s="10"/>
@@ -2093,15 +2257,33 @@
       <c r="V21" s="11"/>
       <c r="W21"/>
       <c r="X21"/>
-      <c r="Y21"/>
-      <c r="Z21" s="10"/>
-      <c r="AA21" s="10"/>
-      <c r="AB21"/>
-      <c r="AC21" s="11"/>
-      <c r="AD21"/>
-      <c r="AE21"/>
-      <c r="AF21"/>
-      <c r="AG21" s="10"/>
+      <c r="Y21" t="s">
+        <v>39</v>
+      </c>
+      <c r="Z21" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AA21" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AC21" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AE21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>39</v>
+      </c>
+      <c r="AG21" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="AH21" s="10"/>
       <c r="AI21"/>
       <c r="AJ21" s="11"/>

</xml_diff>